<commit_message>
Added Library and SCH
</commit_message>
<xml_diff>
--- a/PCB/Library/TemPodLib.xlsx
+++ b/PCB/Library/TemPodLib.xlsx
@@ -1,43 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-21435" yWindow="-10905" windowWidth="21060" windowHeight="14955" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="PartsLibrary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PartsLibrary'!$A$1:$I$1</definedName>
+  </definedNames>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F6FA"/>
+        <bgColor rgb="FFF2F6FA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -45,26 +65,135 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -330,10 +459,198 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="102.5703125" customWidth="1" min="2" max="2"/>
+    <col width="18.28515625" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="39.42578125" customWidth="1" min="6" max="6"/>
+    <col width="48.7109375" customWidth="1" min="7" max="7"/>
+    <col width="46.5703125" customWidth="1" min="8" max="8"/>
+    <col width="117.42578125" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20.1" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>TempMin</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>TempMax</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Library Ref</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Library Path</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Footprint Ref</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Footprint Path</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Datasheet Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ESP32-WROOM-32</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Bluetooth, WiFi 802.11b/g/n, Bluetooth v4.2 +EDR, Class 1, 2 and 3 Transceiver Module U.FL Surface Mount</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>-40</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>85</v>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>ESP32-WROOM-32</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>SCH/ESP32-WROOM-32.SchLib</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>MODULE_ESP32-WROOM-32</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PCB/MODULE_ESP32-WROOM-32.PcbLib</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://documentation.espressif.com/esp32-wroom-32_datasheet_en.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>DHT22</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Digital Relative Humidity &amp; Temperature Sensor, +-2%RH, +-0.5C, Single-Wire Digital Output, 3.3-6V, 4-Pin</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>-40</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>DHT22</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>SCH/DHT22.SchLib</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>DHT22</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>PCB/DHT22.PcbLib</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>https://cdn-shop.adafruit.com/datasheets/Digital+humidity+and+temperature+sensor+AM2302.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1"/>
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1"/>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
+    <row r="12" ht="18" customHeight="1"/>
+    <row r="13" ht="18" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1"/>
+    <row r="15" ht="18" customHeight="1"/>
+    <row r="16" ht="18" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1"/>
+    <row r="20" ht="18" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1"/>
+    <row r="24" ht="18" customHeight="1"/>
+    <row r="25" ht="18" customHeight="1"/>
+    <row r="26" ht="18" customHeight="1"/>
+    <row r="27" ht="18" customHeight="1"/>
+    <row r="28" ht="18" customHeight="1"/>
+    <row r="29" ht="18" customHeight="1"/>
+    <row r="30" ht="18" customHeight="1"/>
+    <row r="31" ht="18" customHeight="1"/>
+    <row r="32" ht="18" customHeight="1"/>
+    <row r="33" ht="18" customHeight="1"/>
+    <row r="34" ht="18" customHeight="1"/>
+    <row r="35" ht="18" customHeight="1"/>
+    <row r="36" ht="18" customHeight="1"/>
+    <row r="37" ht="18" customHeight="1"/>
+    <row r="38" ht="18" customHeight="1"/>
+    <row r="39" ht="18" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1"/>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added battery management component
</commit_message>
<xml_diff>
--- a/PCB/Library/TemPodLib.xlsx
+++ b/PCB/Library/TemPodLib.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -114,6 +114,36 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -476,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -581,138 +611,306 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>DHT22</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>Digital Relative Humidity &amp; Temperature Sensor, +-2%RH, +-0.5C, Single-Wire Digital Output, 3.3-6V, 4-Pin</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n">
+      <c r="C3" s="18" t="n">
         <v>-40</v>
       </c>
-      <c r="D3" s="10" t="n">
+      <c r="D3" s="18" t="n">
         <v>80</v>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>DHT22</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>SCH/DHT22.SchLib</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>DHT22</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>PCB/DHT22.PcbLib</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="19" t="inlineStr">
         <is>
           <t>https://cdn-shop.adafruit.com/datasheets/Digital+humidity+and+temperature+sensor+AM2302.pdf</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>AMS1117-3.3</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>Linearer Spannungsregler, 800 mA, 15 V</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="n">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>AP2112K-3.3</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>600mA CMOS LDO Regulator with Enable, 3.3V Fixed Output, 55uA Iq, SOT-23-5</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="n">
         <v>-40</v>
       </c>
-      <c r="D4" s="10" t="n">
-        <v>125</v>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>AMS1117-3.3</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>SCH/AMS1117-3.3.SchLib</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>SOT229P700X180-4N</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
-        <is>
-          <t>PCB/SOT229P700X180-4N.PcbLib</t>
-        </is>
-      </c>
-      <c r="I4" s="11" t="inlineStr">
-        <is>
-          <t>https://www.snapeda.com/parts/AMS1117-3.3/Advanced%20Monolithic%20Systems/datasheet/</t>
+      <c r="D4" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>AP2112K-3.3TRG1</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>SCH/AP2112K-3P3TRG1.SchLib</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>SOT_RG1_DIO</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>PCB/AP2112K-3P3TRG1.PcbLib</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>https://www.diodes.com/assets/Datasheets/AP2112.pdf</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>AP2112K-3.3</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>600mA CMOS LDO Regulator with Enable, 3.3V Fixed Output, 55uA Iq, SOT-23-5</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="n">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>WeAct 4.2</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>WeAct Studio 4.2in E-Paper Module (400x300, SPI, BWR) interface connector. No dedicated Altium part found online, so implemented as a generic 8-position vertical header matching the module's 8-pin FPC/cable interface, not the module footprint itself.</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="n">
         <v>-40</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>AP2112K-3.3TRG1</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>SCH/AP2112K-3P3TRG1.SchLib</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>SOT_RG1_DIO</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>PCB/AP2112K-3P3TRG1.PcbLib</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>https://www.diodes.com/assets/Datasheets/AP2112.pdf</t>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>WeAct 4.2</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>SCH/WeAct 4.2.SchLib</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>WeAct 4.2</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>PCB/WeAct 4.2.PcbLib</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>https://www.digikey.de/de/models/3068086</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1"/>
-    <row r="7" ht="18" customHeight="1"/>
-    <row r="8" ht="18" customHeight="1"/>
-    <row r="9" ht="18" customHeight="1"/>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>TP4056</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Complete Constant-Current/Constant-Voltage Linear Charger for Single Cell Li-Ion Batteries, 4.2V, up to 1A programmable via resistor, ESOP-8</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>-40</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>TP4056</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>SCH/TP4056.SchLib</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>SOP8-PP_TPW</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>PCB/TP4056.PcbLib</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>https://datasheet.lcsc.com/lcsc/1809261820_TOPPOWER-Nanjing-Extension-Microelectronics-TP4056-42-ESOP8_C16581.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>FS8205A</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Dual N-Channel Enhancement Mode Power MOSFET</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>-55</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>150</v>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>FS8205A</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>SCH/FS8205A.SchLib</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>SOP65P640X120-8N</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>PCB/SOP65P640X120-8N.PcbLib</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>https://www.ic-fortune.com/upload/Download/FS8205A-DS-12_EN.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>DW01A</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>One Cell Lithium-ion/Polymer Battery Protection IC</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>-40</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>DW01A</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>SCH/DW01A.SchLib</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>SOT95P280X145-6N</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>PCB/SOT95P280X145-6N.PcbLib</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>https://www.snapeda.com/parts/DW01A/Fortune%20Semiconductor/datasheet/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Resistor 1206</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Resistor 1206</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>-55</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>125</v>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>SCH/R.SchLib</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>RES1206</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>PCB/Resistor1206.PcbLib</t>
+        </is>
+      </c>
+      <c r="I9" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
     <row r="10" ht="18" customHeight="1"/>
     <row r="11" ht="18" customHeight="1"/>
     <row r="12" ht="18" customHeight="1"/>

</xml_diff>